<commit_message>
Lattice / TA / double-pass AOM baseplates V9.3: no M2.5 in the plate under the TA, tapping sheets
- The TA butterfly board now mounts on the TA adapter (new class
  TA_butterfly_on_adapter in optomech.py). The four M2.5 tapped holes the
  plate carried under the TA are removed from the lattice and TA baseplates;
  the adapter's four 8-32 plate taps stay and the adapter itself is unchanged.
  Plate volume +182.195 mm^3 on both boards, exactly the four 2.05 x 13.8 mm
  bores; nothing else moved and the audits report the same accepted items.
- Lattice and TA baseplate STEPs re-exported; renders, audit reports and BOMs
  regenerated.
- Added *_TAP_or_NOT sheets (PDF + PNG) for the three baseplates and for the
  TA and AOM adapters: which holes are tapped and which are not, nothing else.
- README: V9.3 notes and change log.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DFH1siLiJL3zznbUW9DDQr
</commit_message>
<xml_diff>
--- a/Production/AOMDoublePassV9/AOM_DoublePass_Board_V9.xlsx
+++ b/Production/AOMDoublePassV9/AOM_DoublePass_Board_V9.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="88" customWidth="1" min="1" max="1"/>
@@ -698,26 +698,33 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Counts come from the FreeCAD model (the *_validation.json audit report); adapters are per hana-branch Production/Adapters STEP names.</t>
+          <t>Which holes are tapped and which are not: see the *_TAP_or_NOT sheets next to the STEP file.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>The empty RSP05 mounts on the output rows receive a bonded PBS cube each (not modelled): add 1 cube per "empty rotating PBS RSP05".</t>
+          <t>Counts come from the FreeCAD model (the *_validation.json audit report); adapters are per hana-branch Production/Adapters STEP names.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>HKTS-5/64 adjusters are the two per M05 / KA05T mount (already included with the mounts if bought as kits).</t>
+          <t>The empty RSP05 mounts on the output rows receive a bonded PBS cube each (not modelled): add 1 cube per "empty rotating PBS RSP05".</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
+        <is>
+          <t>HKTS-5/64 adjusters are the two per M05 / KA05T mount (already included with the mounts if bought as kits).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
         <is>
           <t>AOM seats are machined into the baseplate (integral seat, flat screw face); only the upper AOM adapter is a separate part.</t>
         </is>

</xml_diff>